<commit_message>
Actualizar cuentas de formacion (53.215e) y gastos de comerciales con estacionalidad mensual
</commit_message>
<xml_diff>
--- a/Desglose 2027 Presupuestos V5.xlsx
+++ b/Desglose 2027 Presupuestos V5.xlsx
@@ -673,8 +673,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:X206"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:X206"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
@@ -15696,48 +15696,47 @@
         </is>
       </c>
       <c r="K169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="L169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="M169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="N169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="O169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="P169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="Q169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="R169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="S169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="T169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="U169" s="8" t="n">
-        <v>-1846.33</v>
+        <v>-4434.58</v>
       </c>
       <c r="V169" s="8" t="n">
-        <v>-1846.33</v>
-      </c>
-      <c r="W169" s="9">
-        <f>SUM(K169:V169)</f>
-        <v/>
+        <v>-4434.62</v>
+      </c>
+      <c r="W169" s="9" t="n">
+        <v>-53215</v>
       </c>
       <c r="X169" s="10" t="inlineStr">
         <is>
-          <t>Coste operativo general de estructura y servicios de oficinas/fábrica.</t>
+          <t>Presupuesto anual formación no bonificada (53.215,00 €) con reparto mensual lineal homogéneo.</t>
         </is>
       </c>
     </row>
@@ -16056,48 +16055,47 @@
         </is>
       </c>
       <c r="K173" s="8" t="n">
-        <v>-3200</v>
+        <v>-1500</v>
       </c>
       <c r="L173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="M173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="N173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="O173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="P173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="Q173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="R173" s="8" t="n">
-        <v>-3200</v>
+        <v>-1000</v>
       </c>
       <c r="S173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="T173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="U173" s="8" t="n">
-        <v>-3200</v>
+        <v>-2000</v>
       </c>
       <c r="V173" s="8" t="n">
-        <v>-3200</v>
-      </c>
-      <c r="W173" s="9">
-        <f>SUM(K173:V173)</f>
-        <v/>
+        <v>-1500</v>
+      </c>
+      <c r="W173" s="9" t="n">
+        <v>-22000</v>
       </c>
       <c r="X173" s="10" t="inlineStr">
         <is>
-          <t>Gastos comerciales de viaje, kilometraje y dietas vinculados a visitas y prospección de clientes.</t>
+          <t>Gastos comerciales Pere Porta: 2,000.00 €/mes (Agosto al 50%, Enero y Diciembre al 75%). Total año: 22,000.00 €.</t>
         </is>
       </c>
     </row>
@@ -16146,48 +16144,47 @@
         </is>
       </c>
       <c r="K174" s="8" t="n">
-        <v>-2300</v>
+        <v>-1500</v>
       </c>
       <c r="L174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="M174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="N174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="O174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="P174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="Q174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="R174" s="8" t="n">
-        <v>-2300</v>
+        <v>-1000</v>
       </c>
       <c r="S174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="T174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="U174" s="8" t="n">
-        <v>-2300</v>
+        <v>-2000</v>
       </c>
       <c r="V174" s="8" t="n">
-        <v>-2300</v>
-      </c>
-      <c r="W174" s="9">
-        <f>SUM(K174:V174)</f>
-        <v/>
+        <v>-1500</v>
+      </c>
+      <c r="W174" s="9" t="n">
+        <v>-22000</v>
       </c>
       <c r="X174" s="10" t="inlineStr">
         <is>
-          <t>Gastos comerciales de viaje, representación y prospección comercial en zona asignada.</t>
+          <t>Gastos comerciales Ricardo Perez: 2,000.00 €/mes (Agosto al 50%, Enero y Diciembre al 75%). Total año: 22,000.00 €.</t>
         </is>
       </c>
     </row>
@@ -16236,48 +16233,47 @@
         </is>
       </c>
       <c r="K175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-900</v>
       </c>
       <c r="L175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="M175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="N175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="O175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="P175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="Q175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="R175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-600</v>
       </c>
       <c r="S175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="T175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="U175" s="8" t="n">
-        <v>-1092.45</v>
+        <v>-1200</v>
       </c>
       <c r="V175" s="8" t="n">
-        <v>-1092.45</v>
-      </c>
-      <c r="W175" s="9">
-        <f>SUM(K175:V175)</f>
-        <v/>
+        <v>-900</v>
+      </c>
+      <c r="W175" s="9" t="n">
+        <v>-13200</v>
       </c>
       <c r="X175" s="10" t="inlineStr">
         <is>
-          <t>Coste operativo general de estructura y servicios de oficinas/fábrica.</t>
+          <t>Gastos comerciales Javier Paredes: 1,200.00 €/mes (Agosto al 50%, Enero y Diciembre al 75%). Total año: 13,200.00 €.</t>
         </is>
       </c>
     </row>
@@ -16326,48 +16322,47 @@
         </is>
       </c>
       <c r="K176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-1500</v>
       </c>
       <c r="L176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="M176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="N176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="O176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="P176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="Q176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="R176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-1000</v>
       </c>
       <c r="S176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="T176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="U176" s="8" t="n">
-        <v>-800.04</v>
+        <v>-2000</v>
       </c>
       <c r="V176" s="8" t="n">
-        <v>-800.04</v>
-      </c>
-      <c r="W176" s="9">
-        <f>SUM(K176:V176)</f>
-        <v/>
+        <v>-1500</v>
+      </c>
+      <c r="W176" s="9" t="n">
+        <v>-22000</v>
       </c>
       <c r="X176" s="10" t="inlineStr">
         <is>
-          <t>Coste operativo general de estructura y servicios de oficinas/fábrica.</t>
+          <t>Gastos comerciales Garcia: 2,000.00 €/mes (Agosto al 50%, Enero y Diciembre al 75%). Total año: 22,000.00 €.</t>
         </is>
       </c>
     </row>
@@ -16416,48 +16411,47 @@
         </is>
       </c>
       <c r="K177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-450</v>
       </c>
       <c r="L177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="M177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="N177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="O177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="P177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="Q177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="R177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-300</v>
       </c>
       <c r="S177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="T177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="U177" s="8" t="n">
-        <v>-422.84</v>
+        <v>-600</v>
       </c>
       <c r="V177" s="8" t="n">
-        <v>-422.84</v>
-      </c>
-      <c r="W177" s="9">
-        <f>SUM(K177:V177)</f>
-        <v/>
+        <v>-450</v>
+      </c>
+      <c r="W177" s="9" t="n">
+        <v>-6600</v>
       </c>
       <c r="X177" s="10" t="inlineStr">
         <is>
-          <t>Coste operativo general de estructura y servicios de oficinas/fábrica.</t>
+          <t>Gastos comerciales Irene: 600.00 €/mes (Agosto al 50%, Enero y Diciembre al 75%). Total año: 6,600.00 €.</t>
         </is>
       </c>
     </row>
@@ -16686,48 +16680,47 @@
         </is>
       </c>
       <c r="K180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-450</v>
       </c>
       <c r="L180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="M180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="N180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="O180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="P180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="Q180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="R180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-300</v>
       </c>
       <c r="S180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="T180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="U180" s="8" t="n">
-        <v>-141.14</v>
+        <v>-600</v>
       </c>
       <c r="V180" s="8" t="n">
-        <v>-141.14</v>
-      </c>
-      <c r="W180" s="9">
-        <f>SUM(K180:V180)</f>
-        <v/>
+        <v>-450</v>
+      </c>
+      <c r="W180" s="9" t="n">
+        <v>-6600</v>
       </c>
       <c r="X180" s="10" t="inlineStr">
         <is>
-          <t>Coste operativo general de estructura y servicios de oficinas/fábrica.</t>
+          <t>Gastos comerciales Pedro Medina: 600.00 €/mes (Agosto al 50%, Enero y Diciembre al 75%). Total año: 6,600.00 €.</t>
         </is>
       </c>
     </row>
@@ -19086,7 +19079,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B1:I31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
@@ -19638,7 +19631,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B1:H38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
@@ -20769,7 +20762,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B1:V76"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
@@ -26909,7 +26902,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B1:H9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>

</xml_diff>

<commit_message>
Actualizacion pedidos 05.10 comerciales, revisiones Q4 y modulo MRP
</commit_message>
<xml_diff>
--- a/Desglose 2027 Presupuestos V5.xlsx
+++ b/Desglose 2027 Presupuestos V5.xlsx
@@ -673,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X206"/>
+  <dimension ref="B1:X206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -2646,40 +2646,40 @@
         </is>
       </c>
       <c r="K24" s="8" t="n">
-        <v>-247571.61</v>
+        <v>-235193.03</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>-480047.38</v>
+        <v>-456045.01</v>
       </c>
       <c r="M24" s="8" t="n">
-        <v>-505499.75</v>
+        <v>-480224.76</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-391336.67</v>
+        <v>-371769.84</v>
       </c>
       <c r="O24" s="8" t="n">
-        <v>-639721.61</v>
+        <v>-607735.53</v>
       </c>
       <c r="P24" s="8" t="n">
-        <v>-660412.55</v>
+        <v>-627391.92</v>
       </c>
       <c r="Q24" s="8" t="n">
-        <v>-425647.17</v>
+        <v>-404364.81</v>
       </c>
       <c r="R24" s="8" t="n">
-        <v>-255306.21</v>
+        <v>-242540.9</v>
       </c>
       <c r="S24" s="8" t="n">
-        <v>-154533.56</v>
+        <v>-146806.88</v>
       </c>
       <c r="T24" s="8" t="n">
-        <v>-257348.52</v>
+        <v>-244481.09</v>
       </c>
       <c r="U24" s="8" t="n">
-        <v>-410647.96</v>
+        <v>-390115.56</v>
       </c>
       <c r="V24" s="8" t="n">
-        <v>-422003.72</v>
+        <v>-400903.53</v>
       </c>
       <c r="W24" s="9">
         <f>SUM(K24:V24)</f>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="X24" s="10" t="inlineStr">
         <is>
-          <t>Presupuesto de Compras 2027: Materias primas según necesidades netas de formulación industrial (-4.850.076,71 € base; 4.995.578,01 € con reserva MOQ 3%).</t>
+          <t>Presupuesto de Compras 2027: Materias primas proyectadas exclusivamente con la subida del +4,5% por inflación prevista (-4.607.572,86 € base con reserva MOQ 3%).</t>
         </is>
       </c>
     </row>
@@ -2736,40 +2736,40 @@
         </is>
       </c>
       <c r="K25" s="8" t="n">
-        <v>-51110.53</v>
+        <v>-48555</v>
       </c>
       <c r="L25" s="8" t="n">
-        <v>-99104.56</v>
+        <v>-94149.33</v>
       </c>
       <c r="M25" s="8" t="n">
-        <v>-104359.14</v>
+        <v>-99141.17999999999</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>-80790.46000000001</v>
+        <v>-76750.94</v>
       </c>
       <c r="O25" s="8" t="n">
-        <v>-132068.9</v>
+        <v>-125465.45</v>
       </c>
       <c r="P25" s="8" t="n">
-        <v>-136340.49</v>
+        <v>-129523.47</v>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>-87873.77</v>
+        <v>-83480.08</v>
       </c>
       <c r="R25" s="8" t="n">
-        <v>-52707.32</v>
+        <v>-50071.95</v>
       </c>
       <c r="S25" s="8" t="n">
-        <v>-31903.06</v>
+        <v>-30307.91</v>
       </c>
       <c r="T25" s="8" t="n">
-        <v>-53128.95</v>
+        <v>-50472.5</v>
       </c>
       <c r="U25" s="8" t="n">
-        <v>-84777.23</v>
+        <v>-80538.37</v>
       </c>
       <c r="V25" s="8" t="n">
-        <v>-87121.59</v>
+        <v>-82765.50999999999</v>
       </c>
       <c r="W25" s="9">
         <f>SUM(K25:V25)</f>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="X25" s="10" t="inlineStr">
         <is>
-          <t>Presupuesto de Compras 2027: Envases y bidones de envasado (-1.001.286,00 €; 1.031.324,58 € con MOQ 3%).</t>
+          <t>Presupuesto de Compras 2027: Envases y bidones proyectados exclusivamente con +4,5% de inflación (-951.221,69 € con reserva MOQ 3%).</t>
         </is>
       </c>
     </row>
@@ -2916,40 +2916,40 @@
         </is>
       </c>
       <c r="K27" s="8" t="n">
-        <v>-7981.03</v>
+        <v>-7581.98</v>
       </c>
       <c r="L27" s="8" t="n">
-        <v>-15475.42</v>
+        <v>-14701.65</v>
       </c>
       <c r="M27" s="8" t="n">
-        <v>-16295.93</v>
+        <v>-15481.13</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-12615.62</v>
+        <v>-11984.84</v>
       </c>
       <c r="O27" s="8" t="n">
-        <v>-20622.88</v>
+        <v>-19591.74</v>
       </c>
       <c r="P27" s="8" t="n">
-        <v>-21289.9</v>
+        <v>-20225.4</v>
       </c>
       <c r="Q27" s="8" t="n">
-        <v>-13721.7</v>
+        <v>-13035.61</v>
       </c>
       <c r="R27" s="8" t="n">
-        <v>-8230.370000000001</v>
+        <v>-7818.85</v>
       </c>
       <c r="S27" s="8" t="n">
-        <v>-4981.74</v>
+        <v>-4732.65</v>
       </c>
       <c r="T27" s="8" t="n">
-        <v>-8296.209999999999</v>
+        <v>-7881.4</v>
       </c>
       <c r="U27" s="8" t="n">
-        <v>-13238.17</v>
+        <v>-12576.26</v>
       </c>
       <c r="V27" s="8" t="n">
-        <v>-13604.25</v>
+        <v>-12924.04</v>
       </c>
       <c r="W27" s="9">
         <f>SUM(K27:V27)</f>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="X27" s="10" t="inlineStr">
         <is>
-          <t>Presupuesto de Compras 2027: Etiquetas bobina y adhesivas (-156.353,22 €; 161.043,82 € con MOQ 3%).</t>
+          <t>Presupuesto de Compras 2027: Etiquetas bobina y adhesivas proyectadas con +4,5% de inflación (-148.535,55 € con reserva MOQ 3%).</t>
         </is>
       </c>
     </row>
@@ -3006,40 +3006,40 @@
         </is>
       </c>
       <c r="K28" s="8" t="n">
-        <v>-8300.27</v>
+        <v>-7885.26</v>
       </c>
       <c r="L28" s="8" t="n">
-        <v>-16094.43</v>
+        <v>-15289.71</v>
       </c>
       <c r="M28" s="8" t="n">
-        <v>-16947.77</v>
+        <v>-16100.38</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>-13120.25</v>
+        <v>-12464.24</v>
       </c>
       <c r="O28" s="8" t="n">
-        <v>-21447.79</v>
+        <v>-20375.4</v>
       </c>
       <c r="P28" s="8" t="n">
-        <v>-22141.49</v>
+        <v>-21034.42</v>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>-14270.57</v>
+        <v>-13557.04</v>
       </c>
       <c r="R28" s="8" t="n">
-        <v>-8559.59</v>
+        <v>-8131.61</v>
       </c>
       <c r="S28" s="8" t="n">
-        <v>-5181.01</v>
+        <v>-4921.96</v>
       </c>
       <c r="T28" s="8" t="n">
-        <v>-8628.059999999999</v>
+        <v>-8196.66</v>
       </c>
       <c r="U28" s="8" t="n">
-        <v>-13767.69</v>
+        <v>-13079.31</v>
       </c>
       <c r="V28" s="8" t="n">
-        <v>-14148.42</v>
+        <v>-13441</v>
       </c>
       <c r="W28" s="9">
         <f>SUM(K28:V28)</f>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="X28" s="10" t="inlineStr">
         <is>
-          <t>Presupuesto de Compras 2027: Palets homologados nacional y exportación (-162.607,34 €; 167.485,56 € con MOQ 3%).</t>
+          <t>Presupuesto de Compras 2027: Palets homologados proyectados con +4,5% de inflación (-154.476,99 € con reserva MOQ 3%).</t>
         </is>
       </c>
     </row>
@@ -3276,40 +3276,40 @@
         </is>
       </c>
       <c r="K31" s="8" t="n">
-        <v>-4277.83</v>
+        <v>-4063.94</v>
       </c>
       <c r="L31" s="8" t="n">
-        <v>-8294.82</v>
+        <v>-7880.08</v>
       </c>
       <c r="M31" s="8" t="n">
-        <v>-8734.620000000001</v>
+        <v>-8297.889999999999</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>-6761.97</v>
+        <v>-6423.87</v>
       </c>
       <c r="O31" s="8" t="n">
-        <v>-11053.86</v>
+        <v>-10501.17</v>
       </c>
       <c r="P31" s="8" t="n">
-        <v>-11411.38</v>
+        <v>-10840.81</v>
       </c>
       <c r="Q31" s="8" t="n">
-        <v>-7354.83</v>
+        <v>-6987.09</v>
       </c>
       <c r="R31" s="8" t="n">
-        <v>-4411.48</v>
+        <v>-4190.91</v>
       </c>
       <c r="S31" s="8" t="n">
-        <v>-2670.21</v>
+        <v>-2536.7</v>
       </c>
       <c r="T31" s="8" t="n">
-        <v>-4446.77</v>
+        <v>-4224.43</v>
       </c>
       <c r="U31" s="8" t="n">
-        <v>-7095.66</v>
+        <v>-6740.88</v>
       </c>
       <c r="V31" s="8" t="n">
-        <v>-7291.88</v>
+        <v>-6927.29</v>
       </c>
       <c r="W31" s="9">
         <f>SUM(K31:V31)</f>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="X31" s="10" t="inlineStr">
         <is>
-          <t>Presupuesto de Compras 2027: Tapones dosificadores y de seguridad (-83.805,31 €; 86.319,47 € con MOQ 3%).</t>
+          <t>Presupuesto de Compras 2027: Tapones dosificadores proyectados con +4,5% de inflación (-79.615,06 € con reserva MOQ 3%).</t>
         </is>
       </c>
     </row>
@@ -19078,7 +19078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I31"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -19103,6 +19103,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="B4" s="11" t="inlineStr">
         <is>
@@ -19471,6 +19472,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="22" t="inlineStr">
         <is>
@@ -19582,6 +19585,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="B27" s="29" t="inlineStr">
         <is>
@@ -19607,6 +19611,7 @@
       <c r="F29" s="42" t="n"/>
       <c r="G29" s="43" t="n"/>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>

</xml_diff>